<commit_message>
Add Unbedenklichkeitsbescheinigung health insurance status analysis
</commit_message>
<xml_diff>
--- a/00_INBOX - Входящи - Eingang/Accounting_Organized/file_organization_manifest.xlsx
+++ b/00_INBOX - Входящи - Eingang/Accounting_Organized/file_organization_manifest.xlsx
@@ -105,7 +105,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000040773__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000040773.jpg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -192,7 +192,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000040774__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000040774.jpg</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -279,7 +279,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000047298 (1)__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000047298 (1).jpg</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -366,7 +366,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000047301 (1)__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000047301 (1).jpg</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/10001_01-2024_DivAuswertungen_DivMitarbeiter_2Z1 (2)__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/10001_01-2024_DivAuswertungen_DivMitarbeiter_2Z1 (2).pdf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/12-2024_Brutto_Netto_00090_X0B__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/12-2024_Brutto_Netto_00090_X0B.pdf</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Matched keywords: tk, kkh, krankenkasse, sozialversicherung</t>
+          <t>Matched keywords: tk, kkh, krankenkasse, sozialversicherung, bescheinigung</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240105_214356__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240105_214356.jpg</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240118_201244__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240118_201244.jpg</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240118_201333__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240118_201333.jpg</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240122_213234__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240122_213234.jpg</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2217,7 +2217,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240122_213354__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240122_213354.jpg</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240122_213523__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240122_213523.jpg</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240207_175537__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240207_175537.jpg</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240207_175612__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240207_175612.jpg</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_154432__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_154432.jpg</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_160151__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_160151.jpg</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_160355__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_160355.jpg</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_160605__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_160605.jpg</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_160917__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_160917.jpg</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_183313__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240213_183313.jpg</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240228_165447__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240228_165447.jpg</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240308_203211__copy2.mp4</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240308_203211.mp4</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3261,7 +3261,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240308_203259__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240308_203259.jpg</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240313_192946__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240313_192946.jpg</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240313_193308(1)__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240313_193308(1).jpg</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3522,7 +3522,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/20240313_193308__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/20240313_193308.jpg</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240318_074925__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240318_074925.jpg</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240318_174927__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240318_174927.jpg</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240321_074606__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240321_074606.jpg</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240323_055457__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240323_055457.jpg</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3957,7 +3957,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240323_060040__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240323_060040.jpg</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240405_091317__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240405_091317.jpg</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240405_165837__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240405_165837.jpg</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240405_165922__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240405_165922.jpg</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240409_145317__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240409_145317.jpg</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240411_200249__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240411_200249.jpg</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240411_200351__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240411_200351.jpg</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240411_200423__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240411_200423.jpg</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240412_173242__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240412_173242.jpg</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -4740,7 +4740,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240421_160012__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240421_160012.jpg</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -4827,7 +4827,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240425_073935__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240425_073935.jpg</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240503_165138__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240503_165138.jpg</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240503_165410__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240503_165410.jpg</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240506_174920__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240506_174920.jpg</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240513_180215__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240513_180215.jpg</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240518_133837__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240518_133837.jpg</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240525_180048__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240525_180048.jpg</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240603_123040__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240603_123040.jpg</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -5523,7 +5523,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240613_190612__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240613_190612.jpg</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240620_175959__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240620_175959.jpg</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240625_151011__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240625_151011.jpg</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -5784,7 +5784,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240629_074306__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240629_074306.jpg</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -5871,7 +5871,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240703_075444__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240703_075444.jpg</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240725_170837__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240725_170837.jpg</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -6045,7 +6045,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240805_192746__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240805_192746.jpg</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -6132,7 +6132,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240805_193114__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240805_193114.jpg</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240805_193118__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240805_193118.jpg</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240807_150523__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240807_150523.jpg</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240810_105035__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240810_105035.jpg</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -6480,7 +6480,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240908_151654__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240908_151654.jpg</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -6567,7 +6567,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240908_151754__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240908_151754.jpg</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240908_152609__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240908_152609.jpg</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -6741,7 +6741,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240913_133524__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240913_133524.jpg</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240918_170620__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240918_170620.jpg</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -6915,7 +6915,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240929_095748__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240929_095748.jpg</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -7002,7 +7002,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240929_095825__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240929_095825.jpg</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -7089,7 +7089,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240929_100504__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240929_100504.jpg</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -7176,7 +7176,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240929_100825__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240929_100825.jpg</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240930_164727__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20240930_164727.jpg</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -7350,7 +7350,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241003_104857__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241003_104857.jpg</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -7437,7 +7437,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241010_123555__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241010_123555.jpg</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -7524,7 +7524,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241010_124450__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241010_124450.jpg</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241014_155934__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241014_155934.jpg</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -7698,7 +7698,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241127_094823__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241127_094823.jpg</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241212_132952__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241212_132952.jpg</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -7872,7 +7872,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241214_121525__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241214_121525.jpg</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241214_121714__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241214_121714.jpg</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -8046,7 +8046,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241220_033940__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241220_033940.jpg</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -8133,7 +8133,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241224_122812__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20241224_122812.jpg</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250107_102310__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250107_102310.jpg</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -8307,7 +8307,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250110_192304__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250110_192304.jpg</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250113_174639__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250113_174639.jpg</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -8481,7 +8481,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250114_095805__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250114_095805.jpg</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -8568,7 +8568,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250115_195837__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250115_195837.jpg</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -8655,7 +8655,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_160820(1)__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_160820(1).jpg</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -8742,7 +8742,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/20250120_160820__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/20250120_160820.jpg</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -8829,7 +8829,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_160824__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_160824.jpg</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -8916,7 +8916,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250123_111752__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250123_111752.jpg</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250127_151723__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250127_151723.jpg</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -9090,7 +9090,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250212_101528__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250212_101528.jpg</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -9177,7 +9177,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250212_102820__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250212_102820.jpg</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250313_111831__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250313_111831.jpg</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250314_082549__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250314_082549.jpg</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250314_082554__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250314_082554.jpg</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250320_141334__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250320_141334.jpg</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -9612,7 +9612,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250328_160329__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250328_160329.jpg</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250402_095645__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250402_095645.jpg</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -9786,7 +9786,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/307538032__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/307538032.pdf</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -9878,7 +9878,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/02_Payroll/312_neut__Verdienstbescheinigung_Brutto_Netto_01_08_2023_-_31_07_2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/312_neut__Verdienstbescheinigung_Brutto_Netto_01_08_2023_-_31_07_2024.pdf</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -9893,17 +9893,17 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
+          <t>04_Health_Insurance</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
           <t>02_Payroll</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Health Insurance</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -9938,7 +9938,7 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>Matched keywords: brutto_netto</t>
+          <t>Matched keywords: bescheinigung</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -10052,7 +10052,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Aktualisiert- Auszahlungen Inflationsprämie__copy2.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Aktualisiert- Auszahlungen Inflationsprämie.xlsx</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -10139,7 +10139,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/38389 - Vorgangsmappe Lohn - Contributions 28.05.2025__copy2.docx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/38389 - Vorgangsmappe Lohn - Contributions 28.05.2025.docx</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -10333,7 +10333,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -10411,7 +10411,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/42585 - Rechnung 240587_2024 vom 29.06.2024, Aufträge 31_24, 33_23, 33_24, 34_24, Mandant 42303__copy3.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/42585 - Rechnung 240587_2024 vom 29.06.2024, Aufträge 31_24, 33_23, 33_24, 34_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -10431,7 +10431,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_020725__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_020725.pdf</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_040625__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_040625.pdf</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -10695,7 +10695,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_050825__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_050825.pdf</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -10788,7 +10788,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_061224__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_061224.pdf</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -10881,7 +10881,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_070225__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_070225.pdf</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -10974,7 +10974,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_080125__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/6106074_080125.pdf</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/89878877, Antrag auf Ratenzahlung__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/89878877, Antrag auf Ratenzahlung.eml</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -11336,7 +11336,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 01-2025__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 01-2025.eml</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 02-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 02-2024.eml</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -11708,7 +11708,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 02-2025__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 02-2025.eml</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 03-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 03-2024.eml</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -11898,7 +11898,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 04-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 04-2024.eml</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -11994,7 +11994,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 05-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 05-2024.eml</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -12089,7 +12089,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 06-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 06-2024.eml</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -12184,7 +12184,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 07-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 07-2024.eml</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -12279,7 +12279,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 09-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 09-2024.eml</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -12374,7 +12374,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 10-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 10-2024.eml</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -12469,7 +12469,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 11-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 11-2024.eml</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -12564,7 +12564,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 12-2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Accountings 12-2024.eml</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -12658,7 +12658,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/05_Taxes/Anforderung einer regelmäßigen Unbedenklichkeitsbescheinigung im Abonnement.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Anforderung einer regelmäßigen Unbedenklichkeitsbescheinigung im Abonnement.pdf</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -12673,17 +12673,17 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>05_Taxes</t>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>12_Liability_Overview; 04_Health_Insurance; 08_Operating_Costs; 11_Contribution_Lists; 06_Bank_Payments</t>
+          <t>05_Taxes; 12_Liability_Overview; 08_Operating_Costs; 11_Contribution_Lists; 06_Bank_Payments</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Taxes</t>
+          <t>UNBEDENKLICHKEITSBESCHEINIGUNG</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -12723,12 +12723,12 @@
       </c>
       <c r="M144" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>Matched keywords: ust, lst, est</t>
+          <t>Matched keywords: aok, beitragsnachweis, unbedenklichkeitsbescheinigung, unbedenklichkeitsbescheinigungen, bescheinigung, betriebsnummer, Unbedenklichkeitsbescheinigung status document</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
@@ -12755,7 +12755,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Antrag Freischaltung Mein AOK Arbeitgeberservice__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Antrag Freischaltung Mein AOK Arbeitgeberservice.pdf</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -12845,7 +12845,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Aok plus__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Aok plus.eml</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -12938,7 +12938,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Aok Sachsen Anhalt copy document from bank___copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Aok Sachsen Anhalt copy document from bank_.eml</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -13033,7 +13033,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Arbeitsbescheinigung Georgi Stefanov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Arbeitsbescheinigung Georgi Stefanov.pdf</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -13048,7 +13048,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>13_Unknown_To_Review</t>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -13058,7 +13058,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Health Insurance</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -13088,12 +13088,12 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>No category keywords detected.</t>
+          <t>Matched keywords: bescheinigung</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
@@ -13207,7 +13207,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/BKK Linde already clear . I paid__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/BKK Linde already clear . I paid.eml</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -13389,7 +13389,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/bonuses 05_2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/bonuses 05_2024.eml</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -13483,7 +13483,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/bonuses__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/bonuses.eml</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -13570,7 +13570,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20240103_104208_027680__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20240103_104208_027680.pdf</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -13657,7 +13657,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20240516_114103_031693__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20240516_114103_031693.pdf</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -13744,7 +13744,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250106_123149_036763__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250106_123149_036763.pdf</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -13831,7 +13831,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250130_141507_037353__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250130_141507_037353.pdf</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -13918,7 +13918,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250207_104944_037434__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250207_104944_037434.pdf</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250312_121121_038078__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250312_121121_038078.pdf</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -14092,7 +14092,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250425_105744_039055__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20250425_105744_039055.pdf</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -14179,7 +14179,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20251119_133706_044302__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/BRN3C2AF492C3FA_20251119_133706_044302.pdf</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -14354,7 +14354,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/CarlundCarla_RG424005125__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/CarlundCarla_RG424005125.pdf</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -14444,7 +14444,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/CarlundCarla_RG424005157__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/CarlundCarla_RG424005157.pdf</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -14621,7 +14621,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions 03.03.2025__copy2.docx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions 03.03.2025.docx</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -14708,7 +14708,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions 13.03.2025(1)__copy2.docx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions 13.03.2025(1).docx</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -14795,7 +14795,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions 13.03.2025__copy2.docx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions 13.03.2025.docx</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -14882,7 +14882,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions 19.02.2025__copy2.docx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions 19.02.2025.docx</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -14969,7 +14969,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions__copy2.docx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Contributions.docx</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -15056,7 +15056,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/DAK__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/DAK.eml</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Docutain Dokument__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Docutain Dokument.pdf</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -15334,7 +15334,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/enrico_deductions_detailed__copy2.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/enrico_deductions_detailed.xlsx</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -15973,7 +15973,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Favorit MP Martin Zahariev _9005483_vom_04.07.2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Favorit MP Martin Zahariev _9005483_vom_04.07.2025.pdf</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -16065,7 +16065,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 34-2024 Zahariev Martin 04.10.2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 34-2024 Zahariev Martin 04.10.2024.pdf</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -16152,7 +16152,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 71 2025 zahariev Sendungsverlust__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 71 2025 zahariev Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -16242,7 +16242,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Hauptzollamt Erfurt Umbuchung der Zahlung__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Hauptzollamt Erfurt Umbuchung der Zahlung.pdf</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -16329,7 +16329,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Health insurance fund reimbursements__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Health insurance fund reimbursements.eml</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -16422,7 +16422,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Healts Vers.__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Healts Vers..eml</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -16609,7 +16609,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/image__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/image.png</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -16696,7 +16696,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/image001__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/image001.png</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -16783,7 +16783,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/image00122__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/image00122.png</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -16870,7 +16870,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/image222__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/image222.png</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -16957,7 +16957,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/invoices__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/invoices.eml</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -17614,7 +17614,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/KKH(1)__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/KKH(1).eml</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -17702,7 +17702,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/KKH__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/KKH.eml</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -17790,7 +17790,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/KKH1__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/KKH1.eml</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -18755,7 +18755,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Mahnbescheid Amtsgericht Euskirchen _ AXA__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Mahnbescheid Amtsgericht Euskirchen _ AXA.eml</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -18850,7 +18850,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Mahnung Finanzamt__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Mahnung Finanzamt.eml</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -18946,7 +18946,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Martin Zahariev - Bescheid - Adressnachweis__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Martin Zahariev - Bescheid - Adressnachweis.pdf</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -19033,7 +19033,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 51 17.02.2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 51 17.02.2025.pdf</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -19120,7 +19120,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 55 08.03.2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 55 08.03.2025.pdf</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -19295,7 +19295,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/original_msg(1)__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/original_msg(1).eml</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -19391,7 +19391,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/original_msg(2)__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/original_msg(2).eml</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -19484,7 +19484,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/original_msg__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/original_msg.eml</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -19571,7 +19571,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Petya Stefanova AOK__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Petya Stefanova AOK.eml</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -19667,7 +19667,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/PQ__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/PQ.eml</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -19763,7 +19763,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/11_Contribution_Lists/RE-53380_2024 13.08.2024 09_17_16__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/11_Contribution_Lists/RE-53380_2024 13.08.2024 09_17_16.pdf</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -19856,7 +19856,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/11_Contribution_Lists/RE-53652_2024 20.09.2024 10_56_50__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/11_Contribution_Lists/RE-53652_2024 20.09.2024 10_56_50.pdf</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -20215,7 +20215,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Remaining health insurances for 09_2024 und 10_2024__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Remaining health insurances for 09_2024 und 10_2024.eml</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -20610,7 +20610,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>11_Contribution_Lists; 05_Taxes</t>
+          <t>11_Contribution_Lists; 04_Health_Insurance; 05_Taxes</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -20679,7 +20679,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Screenshot_20240212_173450_Samsung Internet__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Screenshot_20240212_173450_Samsung Internet.jpg</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -20766,7 +20766,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Screenshot_20250121_103739_Revolut__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Screenshot_20250121_103739_Revolut.jpg</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -20853,7 +20853,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Screenshot_20250127_123918_Google__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Screenshot_20250127_123918_Google.jpg</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -20940,7 +20940,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Screenshot_20250127_124135_Google__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Screenshot_20250127_124135_Google.jpg</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -21201,7 +21201,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/SEPA List health security__copy3.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/SEPA List health security.pdf</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -21288,7 +21288,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Still missing__copy2.PNG</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Still missing.PNG</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -21375,7 +21375,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Tabelle nach § 175 InsO mit Grund des Bestreitens__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Tabelle nach § 175 InsO mit Grund des Bestreitens.pdf</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -21476,7 +21476,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/tempFileForShare_20250127-132510__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/tempFileForShare_20250127-132510.jpg</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -21650,7 +21650,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/UB__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/UB.pdf</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>Health Insurance</t>
+          <t>UNBEDENKLICHKEITSBESCHEINIGUNG</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
@@ -21710,12 +21710,12 @@
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="N244" t="inlineStr">
         <is>
-          <t>Matched keywords: barmer, krankenkasse, sozialversicherung</t>
+          <t>Matched keywords: barmer, krankenkasse, sozialversicherung, unbedenklichkeitsbescheinigung, bescheinigung, keine beitragsrueckstaende, keine beitragsrückstände, beitragsrueckstaende, beitragsrückstände, sozialversicherungsbeitraege, sozialversicherungsbeiträge, betriebsnummer, Unbedenklichkeitsbescheinigung status document</t>
         </is>
       </c>
       <c r="O244" t="inlineStr">
@@ -21762,7 +21762,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>11_Contribution_Lists; 05_Taxes</t>
+          <t>11_Contribution_Lists; 04_Health_Insurance; 05_Taxes</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -21832,7 +21832,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed__copy3.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed.png</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -21919,7 +21919,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed1__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed1.png</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -22006,7 +22006,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed222__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed222.jpg</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -22093,7 +22093,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed222__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed222.png</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -22180,7 +22180,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed3__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed3.png</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -22267,7 +22267,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed3333333__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed3333333.jpg</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -22354,7 +22354,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed34.22__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/unnamed34.22.png</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -22717,7 +22717,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Unternehmerabrechnung - VP 120-2400001108__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Unternehmerabrechnung - VP 120-2400001108.pdf</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -22995,7 +22995,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Untitled__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Untitled.jpg</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -23369,7 +23369,7 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>11_Contribution_Lists; 01_Accountant_Emails; 06_Bank_Payments; 12_Liability_Overview; 08_Operating_Costs</t>
+          <t>11_Contribution_Lists; 01_Accountant_Emails; 04_Health_Insurance; 06_Bank_Payments; 12_Liability_Overview; 08_Operating_Costs</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
@@ -23440,7 +23440,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/working hours 04.2025(1)__copy2.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/working hours 04.2025(1).xlsx</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -23527,7 +23527,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/working hours 04.2025__copy2.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/working hours 04.2025.xlsx</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -23707,7 +23707,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Zahlungsavis 8345-1440__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Zahlungsavis 8345-1440.pdf</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -23800,7 +23800,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Zoll payment__copy2.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/01_Accountant_Emails/Zoll payment.eml</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -23895,7 +23895,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Без им22е222__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Без им22е222.png</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -23982,7 +23982,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Без име222__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Без име222.png</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -24417,7 +24417,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/aktuelle Unbedenklichkeitsbescheinigungen__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/aktuelle Unbedenklichkeitsbescheinigungen.pdf</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -24442,7 +24442,7 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>Health Insurance</t>
+          <t>UNBEDENKLICHKEITSBESCHEINIGUNG</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
@@ -24486,7 +24486,7 @@
       </c>
       <c r="N275" t="inlineStr">
         <is>
-          <t>Matched keywords: aok, sozialversicherung</t>
+          <t>Matched keywords: aok, sozialversicherung, unbedenklichkeitsbescheinigung, unbedenklichkeitsbescheinigungen, bescheinigung, keine beitragsrueckstaende, keine beitragsrückstände, beitragsrueckstaende, beitragsrückstände, betriebsnummer, Unbedenklichkeitsbescheinigung status document</t>
         </is>
       </c>
       <c r="O275" t="inlineStr">
@@ -24600,7 +24600,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 01-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 01-2024.pdf</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -24620,7 +24620,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -24687,7 +24687,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 02-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 02-2024.pdf</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -24707,7 +24707,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -24774,7 +24774,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 03-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 03-2024.pdf</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -24794,7 +24794,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 04-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 04-2024.pdf</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -24881,7 +24881,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -24948,7 +24948,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 05-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 05-2024.pdf</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -24968,7 +24968,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
@@ -25035,7 +25035,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 06-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 06-2024.pdf</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -25055,7 +25055,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
@@ -25122,7 +25122,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 07-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 07-2024.pdf</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -25142,7 +25142,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
@@ -25209,7 +25209,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 08-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 08-2024.pdf</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -25229,7 +25229,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
@@ -25296,7 +25296,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 09-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 09-2024.pdf</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -25316,7 +25316,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
@@ -25383,7 +25383,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 10-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 10-2024.pdf</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -25403,7 +25403,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
@@ -25470,7 +25470,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 11-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 11-2024.pdf</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -25490,7 +25490,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -25557,7 +25557,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 12-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 12-2024.pdf</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -25577,7 +25577,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 01-2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 01-2025.pdf</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -25664,7 +25664,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -25731,7 +25731,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 02-2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 02-2025.pdf</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -25751,7 +25751,7 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
@@ -25818,7 +25818,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 03-2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 03-2025.pdf</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -25838,7 +25838,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
@@ -25905,7 +25905,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 04-2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 04-2025.pdf</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -25925,7 +25925,7 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
@@ -25992,7 +25992,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 05-2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 05-2025.pdf</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -26012,7 +26012,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -26079,7 +26079,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 06-2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/03_Employee_Payslips/Entgeltbescheinigungen 06-2025.pdf</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -26099,7 +26099,7 @@
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t/>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -26166,7 +26166,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2023__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2023.pdf</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -26253,7 +26253,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2024.pdf</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -26340,7 +26340,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/bankstatementsfrom2022untilnow__copy2.zip</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/bankstatementsfrom2022untilnow.zip</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -26516,7 +26516,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/02-2023 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/02-2023 #9109.pdf</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -26605,7 +26605,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/04-2022 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/04-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -26694,7 +26694,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/07-2022 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/07-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -26756,7 +26756,7 @@
       </c>
       <c r="N301" t="inlineStr">
         <is>
-          <t>Matched keywords: aok, aok plus, tk, techniker, kkh, bkk, viactiv, vivida, krankenkasse, beitragsnachweis</t>
+          <t>Matched keywords: aok, aok plus, tk, techniker, kkh, bkk, viactiv, vivida, krankenkasse, beitragsnachweis, betriebsnummer</t>
         </is>
       </c>
       <c r="O301" t="inlineStr">
@@ -26783,7 +26783,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/10-2022 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/10-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -26872,7 +26872,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/12-2022 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/12-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -27053,7 +27053,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/02-2022 #9109__copy3.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/02-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -27232,7 +27232,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/06-2021 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/06-2021 #9109.pdf</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -27411,7 +27411,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/09-2021 #9109.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/09-2021 #9109.pdf</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -27426,17 +27426,17 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>06_Bank_Payments</t>
+          <t>04_Health_Insurance</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>04_Health_Insurance; 08_Operating_Costs; 05_Taxes; 07_Cash_Payments; 01_Accountant_Emails; 11_Contribution_Lists; 09_Enrico_Forwarded</t>
+          <t>06_Bank_Payments; 08_Operating_Costs; 05_Taxes; 07_Cash_Payments; 01_Accountant_Emails; 11_Contribution_Lists; 09_Enrico_Forwarded</t>
         </is>
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t>Bank Payments</t>
+          <t>Health Insurance</t>
         </is>
       </c>
       <c r="H309" t="inlineStr">
@@ -27474,7 +27474,7 @@
       </c>
       <c r="N309" t="inlineStr">
         <is>
-          <t>Matched keywords: konto, ueberweisung, überweisung, lastschrift, bank</t>
+          <t>Matched keywords: aok, aok plus, tk, techniker, kkh, bkk, vivida, krankenkasse, betriebsnummer</t>
         </is>
       </c>
       <c r="O309" t="inlineStr">
@@ -27680,7 +27680,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Atanas Madzharov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Atanas Madzharov.pdf</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -27767,7 +27767,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Boris Parvanov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Boris Parvanov.pdf</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -27854,7 +27854,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Boyko Bogdanov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Boyko Bogdanov.pdf</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -27941,7 +27941,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Bozhidar Asenov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Bozhidar Asenov.pdf</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -28028,7 +28028,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Martin Tanev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Martin Tanev.pdf</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -28115,7 +28115,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Nikolay Metodiev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Nikolay Metodiev.pdf</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -28202,7 +28202,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Nikolay Nikolov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Nikolay Nikolov.pdf</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -28289,7 +28289,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Todor Kitanov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Todor Kitanov.pdf</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -28376,7 +28376,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/01-2023 #9120__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/01-2023 #9120.pdf</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -28464,7 +28464,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/02-2022 #9109__copy4.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/02-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -28644,7 +28644,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/02-2023 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/02-2023 #9109.pdf</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -28733,7 +28733,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/03-2023 #9120__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/03-2023 #9120.pdf</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -28822,7 +28822,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/04-2022 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/04-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -29002,7 +29002,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/06-2022 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/06-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -29064,7 +29064,7 @@
       </c>
       <c r="N327" t="inlineStr">
         <is>
-          <t>Matched keywords: aok, aok plus, tk, techniker, kkh, bkk, viactiv, vivida, krankenkasse, beitragsnachweis, Hauptzollamt related to Krankenkasse</t>
+          <t>Matched keywords: aok, aok plus, tk, techniker, kkh, bkk, viactiv, vivida, krankenkasse, beitragsnachweis, betriebsnummer, Hauptzollamt related to Krankenkasse</t>
         </is>
       </c>
       <c r="O327" t="inlineStr">
@@ -29182,7 +29182,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/07-2022 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/07-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -29360,7 +29360,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/10-2022 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/10-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -29538,7 +29538,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/12-2022 #9109__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/12-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -29720,7 +29720,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/501 - Boryana Trichkova__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/501 - Boryana Trichkova.pdf</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -29807,7 +29807,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/502 - Darin Veselinov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/502 - Darin Veselinov.pdf</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -29894,7 +29894,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/503 - Petar Genov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/503 - Petar Genov.pdf</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -29981,7 +29981,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/509 - Ivan Ivanov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/509 - Ivan Ivanov.pdf</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -30068,7 +30068,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/513 - Nikolay Nikolov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/513 - Nikolay Nikolov.pdf</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -30155,7 +30155,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/516 - Miroslav Milovoev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/516 - Miroslav Milovoev.pdf</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -30242,7 +30242,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/517 - Kiril Nikolov__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/517 - Kiril Nikolov.pdf</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -30329,7 +30329,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Boyko Bogdanov - 062021 Erhalten in bar__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Boyko Bogdanov - 062021 Erhalten in bar.pdf</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -30416,7 +30416,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Todor Kitanov - 062021 Erhalten in bar__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Todor Kitanov - 062021 Erhalten in bar.pdf</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -31025,7 +31025,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/a_002__copy2.htm</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/a_002.htm</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -34274,7 +34274,7 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
@@ -34467,7 +34467,7 @@
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
@@ -34660,7 +34660,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>01_Accountant_Emails; 11_Contribution_Lists; 05_Taxes; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>01_Accountant_Emails; 11_Contribution_Lists; 05_Taxes; 06_Bank_Payments; 03_Employee_Payslips; 04_Health_Insurance; 02_Payroll</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -34853,7 +34853,7 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
@@ -34931,7 +34931,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Accountings 03-2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Accountings 03-2024.pdf</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -35038,7 +35038,7 @@
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -35211,7 +35211,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/42585 - Rechnung 240587_2024 vom 29.06.2024, Aufträge 31_24, 33_23, 33_24, 34_24, Mandant 42303__copy4.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/42585 - Rechnung 240587_2024 vom 29.06.2024, Aufträge 31_24, 33_23, 33_24, 34_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
@@ -35231,7 +35231,7 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
@@ -35617,7 +35617,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
@@ -35810,7 +35810,7 @@
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
@@ -36196,7 +36196,7 @@
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
@@ -36753,7 +36753,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/40579 - Rechnung 240155_2024 vom 17.02.2024, Aufträge 31_23, 33_23, 34_23, Mandant 42303__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/40579 - Rechnung 240155_2024 vom 17.02.2024, Aufträge 31_23, 33_23, 34_23, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -36870,7 +36870,7 @@
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 03_Employee_Payslips; 02_Payroll</t>
+          <t>05_Taxes; 01_Accountant_Emails; 11_Contribution_Lists; 06_Bank_Payments; 04_Health_Insurance; 03_Employee_Payslips; 02_Payroll</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
@@ -37652,7 +37652,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2023__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2023.pdf</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -37739,7 +37739,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2024.pdf</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -37913,7 +37913,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/9. Nachweise zur Anmeldung der Mitarbeiter beim Sozialversicherungsträger__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/9. Nachweise zur Anmeldung der Mitarbeiter beim Sozialversicherungsträger.pdf</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -38087,7 +38087,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie__copy4.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie.xlsx</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -38174,7 +38174,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Working Hours 04.2024__copy2.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/Working Hours 04.2024.xlsx</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -38348,7 +38348,7 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie__copy5.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie__copy2.xlsx</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -38435,7 +38435,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Working Hours 03-2024 __copy2.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Working Hours 03-2024 .xlsx</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
@@ -38522,7 +38522,7 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/10001_00069_Turchalieva_Maria_Desislava_07_2024_Div_Auswertungen_I03 (1)__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/10001_00069_Turchalieva_Maria_Desislava_07_2024_Div_Auswertungen_I03 (1).pdf</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
@@ -38609,7 +38609,7 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/10001_00070_Stefanova_Petya_06_2024_Div_Auswertungen_F0B__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/10001_00070_Stefanova_Petya_06_2024_Div_Auswertungen_F0B.pdf</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -38870,7 +38870,7 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_162838__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_162838.jpg</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
@@ -38957,7 +38957,7 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_162844__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_162844.jpg</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
@@ -39044,7 +39044,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_162848__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/20250120_162848.jpg</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
@@ -39131,7 +39131,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 66 Mai 2025 zahariev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 66 Mai 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -39219,7 +39219,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Mai 25 Sachsenpower GmbH &amp; Co. KG__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Mai 25 Sachsenpower GmbH &amp; Co. KG.pdf</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -39308,7 +39308,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 31-2024 Zahariev Martin 30.09.2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 31-2024 Zahariev Martin 30.09.2024.pdf</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -39396,7 +39396,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis September 2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis September 2024.pdf</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -39661,7 +39661,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 05.04. 2025 zahariev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 05.04. 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -39751,7 +39751,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2764 Zahariev Hermes Kleidung__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2764 Zahariev Hermes Kleidung.pdf</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -39929,7 +39929,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2766 Zahariev Hermes Sendungsverlust__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2766 Zahariev Hermes Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -40022,7 +40022,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2767 Zahariev Hermes Bearbeitungsgebuhr__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2767 Zahariev Hermes Bearbeitungsgebuhr.pdf</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -40112,7 +40112,7 @@
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/gutschrift 66 Mai 2025 zahariev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/gutschrift 66 Mai 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -40200,7 +40200,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/gutschrift 71 2025 zahariev Sendungsverlust__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/gutschrift 71 2025 zahariev Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
@@ -40468,7 +40468,7 @@
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2794 Zahariev KFZ Miete__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2794 Zahariev KFZ Miete.pdf</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
@@ -40556,7 +40556,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2798 Zahariev Hermes Sendungsverlust__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2798 Zahariev Hermes Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
@@ -40738,7 +40738,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 42-2024 Zahariev Martin 30.11.2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 42-2024 Zahariev Martin 30.11.2024.pdf</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -40826,7 +40826,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2014 vom 05.12.2024 Sendungsverlust Zahariev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2014 vom 05.12.2024 Sendungsverlust Zahariev.pdf</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -40919,7 +40919,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2015 07.12.2024 Martin Zahariev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2015 07.12.2024 Martin Zahariev.pdf</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
@@ -41007,7 +41007,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2023 vom 07.12.2024  Zahariev HERMES Bekleidung__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2023 vom 07.12.2024  Zahariev HERMES Bekleidung.pdf</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
@@ -41549,7 +41549,7 @@
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/2022 Arbeitgeberbestätigung zu den Arbeitstagen__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/2022 Arbeitgeberbestätigung zu den Arbeitstagen.pdf</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
@@ -41637,7 +41637,7 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/2023 Arbeitgeberbestätigung zu den Arbeitstagen__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/2023 Arbeitgeberbestätigung zu den Arbeitstagen.pdf</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
@@ -41725,7 +41725,7 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000038649 (1)__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000038649 (1).jpg</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
@@ -41812,7 +41812,7 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000038651__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000038651.jpg</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
@@ -41899,7 +41899,7 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000038655__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000038655.jpg</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
@@ -41986,7 +41986,7 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000038657__copy2.jpg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/1000038657.jpg</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
@@ -42247,7 +42247,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 38-2024 Zahariev Martin 31.10.2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 38-2024 Zahariev Martin 31.10.2024.pdf</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
@@ -42335,7 +42335,7 @@
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Oktober 2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Oktober 2024.pdf</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
@@ -42424,7 +42424,7 @@
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Gutschrift 42-2024 Zahariev Martin 30.11.2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Gutschrift 42-2024 Zahariev Martin 30.11.2024.pdf</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
@@ -42512,7 +42512,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis November 2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis November 2024.pdf</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
@@ -42601,7 +42601,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 44-2024 Zahariev Martin 31.12.2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 44-2024 Zahariev Martin 31.12.2024.pdf</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
@@ -42689,7 +42689,7 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Dezember Zahariev 2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Dezember Zahariev 2024.pdf</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
@@ -42778,7 +42778,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift April 2025 zahariev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift April 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
@@ -42866,7 +42866,7 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev April 25 Sachsenpower GmbH &amp; Co. KG__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev April 25 Sachsenpower GmbH &amp; Co. KG.pdf</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
@@ -42955,7 +42955,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift märz 2025 zahariev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift märz 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
@@ -43042,7 +43042,7 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Subunternehmer Sachsenpower GmbH &amp; Co. KG__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Subunternehmer Sachsenpower GmbH &amp; Co. KG.pdf</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
@@ -43131,7 +43131,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Martin Zahariev Februar 2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Martin Zahariev Februar 2025.pdf</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
@@ -43220,7 +43220,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 52 28.02.2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 52 28.02.2025.pdf</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
@@ -43308,7 +43308,7 @@
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 24-2024 Zahariev Martin 31.07.2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 24-2024 Zahariev Martin 31.07.2024.pdf</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
@@ -43396,7 +43396,7 @@
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Juli 2024__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Juli 2024.pdf</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
@@ -43485,7 +43485,7 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift Zahariev 74 30.06.2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift Zahariev 74 30.06.2025.pdf</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
@@ -43573,7 +43573,7 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Juni 25 Sachsenpower GmbH &amp; Co. KG__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Juni 25 Sachsenpower GmbH &amp; Co. KG.pdf</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
@@ -43662,7 +43662,7 @@
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Martin Zahariev Januar 2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Martin Zahariev Januar 2025.pdf</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
@@ -43751,7 +43751,7 @@
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 48 31.01.2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 48 31.01.2025.pdf</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
@@ -43839,7 +43839,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2035 08.01.2025 Hermes Bekleidung__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2035 08.01.2025 Hermes Bekleidung.pdf</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
@@ -44107,7 +44107,7 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2038 08.01.2025 Bearbeitungsgebühr__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2038 08.01.2025 Bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
@@ -44376,7 +44376,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2056 07.02.2025 Bearbeitungsgebühr__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2056 07.02.2025 Bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
@@ -44464,7 +44464,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2057 07.02.2025 Hermes Bekleidung__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2057 07.02.2025 Hermes Bekleidung.pdf</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
@@ -44551,7 +44551,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/image222__copy2.png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/image222.png</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
@@ -44638,7 +44638,7 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2069 08.03.2025 Sendungsverluste__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2069 08.03.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
@@ -44726,7 +44726,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2070 08.03.2025 Sendungsverluste__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2070 08.03.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
@@ -44814,7 +44814,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/unnamed34__copy2.22png</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/unnamed34.22png</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
@@ -45079,7 +45079,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2781 Zahariev Hermes Sendungsverlust__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2781 Zahariev Hermes Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
@@ -45614,7 +45614,7 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2812 Zahariev Hermes Sendungsverlust__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2812 Zahariev Hermes Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
@@ -45977,7 +45977,7 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Rechnung 2788 Zahariev Hermes Scannermiete__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Rechnung 2788 Zahariev Hermes Scannermiete.pdf</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
@@ -46067,7 +46067,7 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Rechnung 2794 Zahariev KFZ Miete__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Rechnung 2794 Zahariev KFZ Miete.pdf</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
@@ -46155,7 +46155,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Rechnung 2798 Zahariev Hermes Sendungsverlust__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Rechnung 2798 Zahariev Hermes Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
@@ -46247,7 +46247,7 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Rechnung 2799 Bearbeitungsgebühr 10.06.2025 Zahariev__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Rechnung 2799 Bearbeitungsgebühr 10.06.2025 Zahariev.pdf</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
@@ -46518,7 +46518,7 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy19.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen.pdf</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
@@ -47127,7 +47127,7 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy20.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy2.pdf</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
@@ -47301,7 +47301,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy21.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy3.pdf</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
@@ -47475,7 +47475,7 @@
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy22.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy4.pdf</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
@@ -47649,7 +47649,7 @@
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy23.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy5.pdf</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
@@ -47736,7 +47736,7 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie__copy2.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie.xlsx</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
@@ -47910,7 +47910,7 @@
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy24.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy6.pdf</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
@@ -48258,7 +48258,7 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy25.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy7.pdf</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
@@ -48345,7 +48345,7 @@
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy26.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy8.pdf</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
@@ -48800,7 +48800,7 @@
       </c>
       <c r="F549" t="inlineStr">
         <is>
-          <t>02_Payroll; 08_Operating_Costs; 11_Contribution_Lists; 04_Health_Insurance</t>
+          <t>02_Payroll; 04_Health_Insurance; 08_Operating_Costs; 11_Contribution_Lists</t>
         </is>
       </c>
       <c r="G549" t="inlineStr">
@@ -48876,7 +48876,7 @@
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy27.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy9.pdf</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
@@ -48963,7 +48963,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy28.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy10.pdf</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
@@ -49572,7 +49572,7 @@
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Abstimmliste (DE - SEPA, Langform) (3) (1)__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Abstimmliste (DE - SEPA, Langform) (3) (1).pdf</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
@@ -49746,7 +49746,7 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy29.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy11.pdf</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
@@ -49920,7 +49920,7 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy30.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy12.pdf</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
@@ -50007,7 +50007,7 @@
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/SEPA List health security__copy4.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/SEPA List health security.pdf</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
@@ -50355,7 +50355,7 @@
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy31.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy13.pdf</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
@@ -50790,7 +50790,7 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy32.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy14.pdf</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
@@ -51138,7 +51138,7 @@
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy33.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy15.pdf</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
@@ -51225,7 +51225,7 @@
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy34.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy16.pdf</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
@@ -51834,7 +51834,7 @@
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy35.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy17.pdf</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
@@ -51921,7 +51921,7 @@
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy36.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/Lohnauswertungen__copy18.pdf</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
@@ -52443,7 +52443,7 @@
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/IMG-20240531-WA0000__copy2.jpeg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/IMG-20240531-WA0000.jpeg</t>
         </is>
       </c>
       <c r="C591" t="inlineStr">
@@ -52530,7 +52530,7 @@
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/IMG-20240531-WA0002__copy2.jpeg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/IMG-20240531-WA0002.jpeg</t>
         </is>
       </c>
       <c r="C592" t="inlineStr">
@@ -52617,7 +52617,7 @@
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/IMG-20240531-WA0004__copy2.jpeg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/IMG-20240531-WA0004.jpeg</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
@@ -52704,7 +52704,7 @@
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/IMG-20240531-WA0006__copy2.jpeg</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/IMG-20240531-WA0006.jpeg</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
@@ -53139,7 +53139,7 @@
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/2022 ArbeitgeberbestÃ¤tigung zu den Arbeitstagen__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/2022 ArbeitgeberbestÃ¤tigung zu den Arbeitstagen.pdf</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
@@ -53227,7 +53227,7 @@
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/2023 ArbeitgeberbestÃ¤tigung zu den Arbeitstagen__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/14_Duplicates/2023 ArbeitgeberbestÃ¤tigung zu den Arbeitstagen.pdf</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
@@ -53315,7 +53315,7 @@
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/02_Payroll/Lohnauswertungen_März_2025__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/02_Payroll/Lohnauswertungen_März_2025.pdf</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
@@ -53663,7 +53663,7 @@
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie__copy6.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie__copy3.xlsx</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
@@ -53750,7 +53750,7 @@
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/working hours 05.2024__copy2.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/13_Unknown_To_Review/working hours 05.2024.xlsx</t>
         </is>
       </c>
       <c r="C606" t="inlineStr">
@@ -53837,7 +53837,7 @@
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/20240123_60222_10160_Rechnung__copy2.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/20240123_60222_10160_Rechnung.pdf</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
@@ -53950,7 +53950,7 @@
       </c>
       <c r="F608" t="inlineStr">
         <is>
-          <t>05_Taxes; 12_Liability_Overview</t>
+          <t>04_Health_Insurance; 05_Taxes; 12_Liability_Overview</t>
         </is>
       </c>
       <c r="G608" t="inlineStr">

</xml_diff>